<commit_message>
[ROS-LL-v4.1.0] Correct metadata and reference links
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-LL/v4.1.0/Form-ROS-LL-v4.1.0.xlsx
+++ b/form_reporting_templates/ROS-LL/v4.1.0/Form-ROS-LL-v4.1.0.xlsx
@@ -1973,8 +1973,10 @@
       <c r="F4" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="G4" s="8" t="s">
-        <v>253</v>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>4.1.0</t>
+        </is>
       </c>
       <c r="H4" s="9"/>
     </row>
@@ -10326,7 +10328,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1" location="baitSpecies" xr:uid="{D849EFD5-707B-4C7E-BB2A-B091E478F30F}"/>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{D849EFD5-707B-4C7E-BB2A-B091E478F30F}" location="baitSpecies"/>
     <hyperlink ref="C2" r:id="rId2" location="baitConditions" xr:uid="{677A485E-282F-407D-9CFC-1AB91778C9AC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18232,7 +18234,7 @@
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" location="weightMeasurements" xr:uid="{779410D5-0433-4C34-84B6-98A10CA2B249}"/>
     <hyperlink ref="K2" r:id="rId2" location="weightMeasurementTools" xr:uid="{EB80831C-DDCE-4E4D-A605-160D23E19E90}"/>
-    <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}"/>
+    <hyperlink ref="E2" r:id="rId3" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}" location="fateTypes"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{5DE917A8-1BC5-48A5-BE95-3206B5EEB7AC}"/>
     <hyperlink ref="D1" r:id="rId5" location="allSpecies" xr:uid="{7915C09B-5FFF-4B7E-84FB-D8B7D31EA643}"/>
     <hyperlink ref="G1:G2" r:id="rId6" location="samplingMethodsForCatchEstimation" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
@@ -23409,13 +23411,13 @@
   <hyperlinks>
     <hyperlink ref="E1:E2" r:id="rId1" location="samplingPeriods" display="SAMPLING_PERIOD" xr:uid="{C0407D03-A3E9-4479-BB66-8329070009A1}"/>
     <hyperlink ref="V2" r:id="rId2" location="depredationSources" xr:uid="{5248D097-7FB7-4BF7-908D-893A3BF91D4F}"/>
-    <hyperlink ref="W2" r:id="rId3" location="predators" xr:uid="{16A7B676-4806-46E0-B05E-266794DC9A6F}"/>
-    <hyperlink ref="F1:F2" r:id="rId4" location="samplingMethodsForSamplingCollection" display="SAMPLING_METHOD" xr:uid="{863AF79D-449A-4B35-AC8D-9C415D8A32B9}"/>
+    <hyperlink ref="W2" r:id="rId3" xr:uid="{16A7B676-4806-46E0-B05E-266794DC9A6F}" location="predatorSpecies"/>
+    <hyperlink ref="F1:F2" r:id="rId4" display="SAMPLING_METHOD" xr:uid="{863AF79D-449A-4B35-AC8D-9C415D8A32B9}" location="samplingMethodsForSamplingCollections"/>
     <hyperlink ref="I2" r:id="rId5" location="lengthMeasurementTools" xr:uid="{776CD30A-4D78-4230-9891-093ADBA1D96D}"/>
     <hyperlink ref="L2" r:id="rId6" location="lengthMeasurementTools" xr:uid="{3DE19339-45B9-47B8-B5FB-D4012AD9C532}"/>
-    <hyperlink ref="G2" r:id="rId7" location="lengthMeasurementTypes" xr:uid="{4F273766-A7DB-428C-A222-09DB4E6495A6}"/>
+    <hyperlink ref="G2" r:id="rId7" xr:uid="{4F273766-A7DB-428C-A222-09DB4E6495A6}" location="allMeasurements"/>
     <hyperlink ref="J2" r:id="rId8" location="lengthMeasurements" xr:uid="{50D5D995-3D3B-46CA-9856-C3BF09F867B6}"/>
-    <hyperlink ref="O2" r:id="rId9" location="weightEstimationMethods" xr:uid="{6830A97A-B177-4E61-8434-B97D80589AB0}"/>
+    <hyperlink ref="O2" r:id="rId9" xr:uid="{6830A97A-B177-4E61-8434-B97D80589AB0}" location="weightMeasurementTools"/>
     <hyperlink ref="M2" r:id="rId10" location="fishProcessingTypes" xr:uid="{4C80F85B-DC5E-4379-AEDD-32355F2C04AE}"/>
     <hyperlink ref="P1:P2" r:id="rId11" location="sex" display="SEX" xr:uid="{06582CBC-0354-4030-B121-DACE171DCC1B}"/>
     <hyperlink ref="S2" r:id="rId12" location="biologicalMaterials" xr:uid="{66503A95-2496-4FEA-BFDB-8687AAF0A03C}"/>
@@ -27971,16 +27973,16 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="G1:G2" r:id="rId1" location="gearInteractions" display="GEAR_INTERACTION" xr:uid="{4D21FAB4-D1ED-49FA-A8E9-1A452DA8E255}"/>
-    <hyperlink ref="H1:H2" r:id="rId2" location="hookTypes" display="HOOK_TYPE" xr:uid="{FC3E5B48-31F4-4395-B266-CAE8F0285CBE}"/>
+    <hyperlink ref="H1:H2" r:id="rId2" display="HOOK_TYPE" xr:uid="{FC3E5B48-31F4-4395-B266-CAE8F0285CBE}" location="hookAndTerminalDevices"/>
     <hyperlink ref="I2" r:id="rId3" location="baitConditions" xr:uid="{A5E5073A-7EA6-4050-99BD-3A2C3C210913}"/>
     <hyperlink ref="M1:M2" r:id="rId4" location="dehookerTypes" display="DEHOOKER_DEVICE" xr:uid="{223FF70D-0F50-400C-91DF-40947EEFC402}"/>
     <hyperlink ref="K2" r:id="rId5" location="lineMaterialTypes" xr:uid="{8BD5CD8E-6908-4DE0-9B07-7CCA6FB5C649}"/>
     <hyperlink ref="P1:P2" r:id="rId6" location="handlingMethods" display="HANDLING_METHOD" xr:uid="{4AAC5290-0C1E-413E-9063-304F215E9866}"/>
     <hyperlink ref="J2" r:id="rId7" location="baitTypes" xr:uid="{8E341D36-948A-422D-9D66-B4F0241035EC}"/>
-    <hyperlink ref="E1" r:id="rId8" location="individualConditions" display="CONDITION_AT_CAPTURE_CODE" xr:uid="{26B5C55C-6931-4D84-B6B4-4AA585019D2E}"/>
-    <hyperlink ref="F1" r:id="rId9" location="individualConditions" display="CONDITION_AT_RELEASE_CODE" xr:uid="{312D6457-0D67-4610-B478-F5AE649B98F6}"/>
+    <hyperlink ref="E1" r:id="rId8" display="CONDITION_AT_CAPTURE_CODE" xr:uid="{26B5C55C-6931-4D84-B6B4-4AA585019D2E}" location="individualConditions"/>
+    <hyperlink ref="F1" r:id="rId9" display="CONDITION_AT_RELEASE_CODE" xr:uid="{312D6457-0D67-4610-B478-F5AE649B98F6}" location="individualConditions"/>
     <hyperlink ref="S2" r:id="rId10" location="depredationSources" xr:uid="{11FAA504-1FFB-4306-A7A1-4F548FAD3A87}"/>
-    <hyperlink ref="T2" r:id="rId11" location="predators" xr:uid="{AD1EB751-9874-431A-A9CC-CB89B7E2E48C}"/>
+    <hyperlink ref="T2" r:id="rId11" xr:uid="{AD1EB751-9874-431A-A9CC-CB89B7E2E48C}" location="predatorSpecies"/>
     <hyperlink ref="F1:F2" r:id="rId12" location="individualConditions" display="CONDITION_AT_RELEASE" xr:uid="{7022269F-0B3D-487B-821A-D8677291ECA9}"/>
     <hyperlink ref="E1:E2" r:id="rId13" location="individualConditions" display="CONDITION_AT_CAPTURE" xr:uid="{46C1F397-FDC9-4F56-B765-948CEB3929A4}"/>
   </hyperlinks>
@@ -36071,8 +36073,8 @@
     <hyperlink ref="V4" r:id="rId4" location="reasonsDaysLost" xr:uid="{3955310B-45A1-4FFC-AD47-D85E65B9B8C5}"/>
     <hyperlink ref="W4" r:id="rId5" location="reasonsDaysLost" xr:uid="{F6A2D174-87CA-4A84-A59B-9C5B3EDFA410}"/>
     <hyperlink ref="X4" r:id="rId6" location="reasonsDaysLost" xr:uid="{4AD9F6B4-F493-4D51-A425-E40A5E342DD0}"/>
-    <hyperlink ref="E4" r:id="rId7" location="Ports" xr:uid="{8E8691ED-310C-4B0D-98E7-1C757A32EA68}"/>
-    <hyperlink ref="J4" r:id="rId8" location="Ports" xr:uid="{FDCA5CD8-C8A1-4C49-864F-2B6D02C8EA6C}"/>
+    <hyperlink ref="E4" r:id="rId7" xr:uid="{8E8691ED-310C-4B0D-98E7-1C757A32EA68}" location="ports"/>
+    <hyperlink ref="J4" r:id="rId8" xr:uid="{FDCA5CD8-C8A1-4C49-864F-2B6D02C8EA6C}" location="ports"/>
   </hyperlinks>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
@@ -39831,12 +39833,12 @@
   <hyperlinks>
     <hyperlink ref="C2:C3" r:id="rId1" location="countries" display="FLAG_OR_CHARTERING_STATE" xr:uid="{DA9CE3B1-74F9-4268-98AF-290FAC660EAD}"/>
     <hyperlink ref="G2" r:id="rId2" location="countries" display="COUNTRY_CODE" xr:uid="{4939BF01-E483-4611-A010-33B090D54E39}"/>
-    <hyperlink ref="J1" r:id="rId3" location="targetSpecies" display="SPECIES_1_CODE" xr:uid="{E9AF38ED-FD60-4672-8F14-35015A129362}"/>
+    <hyperlink ref="J1" r:id="rId3" display="SPECIES_1_CODE" xr:uid="{E9AF38ED-FD60-4672-8F14-35015A129362}" location="targetSpecies"/>
     <hyperlink ref="M3" r:id="rId4" location="countries" xr:uid="{10913ED0-4328-48D4-A042-6201D824CECA}"/>
     <hyperlink ref="O3" r:id="rId5" location="countries" xr:uid="{3CF4C3FC-91EE-45A1-9C82-1871A741D19A}"/>
-    <hyperlink ref="H2" r:id="rId6" display="PORT_CODE" xr:uid="{C4D05E8A-B26C-4196-BF44-6883318591EB}"/>
+    <hyperlink ref="H2" r:id="rId6" display="PORT_CODE" xr:uid="{C4D05E8A-B26C-4196-BF44-6883318591EB}" location="ports"/>
     <hyperlink ref="K2:K3" r:id="rId7" location="gears" display="MAIN_FISHING_GEAR" xr:uid="{ADDD99C7-B692-4517-AF11-C5F4715C3781}"/>
-    <hyperlink ref="H2:H3" r:id="rId8" location="Ports" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}"/>
+    <hyperlink ref="H2:H3" r:id="rId8" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}" location="ports"/>
     <hyperlink ref="J1:J3" r:id="rId9" location="targetSpecies" display="LICENSED_TARGET_SPECIES" xr:uid="{8145BEA5-06D1-4F1F-890E-1ACE66463F94}"/>
     <hyperlink ref="G2:G3" r:id="rId10" location="countries" display="COUNTRY" xr:uid="{40B25D40-1383-402F-BBDE-DC1B90768417}"/>
   </hyperlinks>
@@ -42553,8 +42555,8 @@
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" location="countries" xr:uid="{D6E7062F-2D43-4596-8E73-CC2381D61A2B}"/>
     <hyperlink ref="G3" r:id="rId2" location="countries" xr:uid="{DE99A7AA-576F-4966-8C9A-C1F406C63AE0}"/>
-    <hyperlink ref="C3" r:id="rId3" location="Ports" xr:uid="{93F08CEF-34DB-46A0-A09B-203AF008B136}"/>
-    <hyperlink ref="H3" r:id="rId4" location="Ports" xr:uid="{2CDE38A1-7DD3-42DB-B597-7777F42628DA}"/>
+    <hyperlink ref="C3" r:id="rId3" xr:uid="{93F08CEF-34DB-46A0-A09B-203AF008B136}" location="ports"/>
+    <hyperlink ref="H3" r:id="rId4" xr:uid="{2CDE38A1-7DD3-42DB-B597-7777F42628DA}" location="ports"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -51482,7 +51484,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D2:D3" r:id="rId1" location="hullMaterialTypes" display="HULL_MATERIAL" xr:uid="{67410786-49B8-4FAC-82C7-693110607986}"/>
+    <hyperlink ref="D2:D3" r:id="rId1" display="HULL_MATERIAL" xr:uid="{67410786-49B8-4FAC-82C7-693110607986}" location="hullMaterialTypes"/>
     <hyperlink ref="L3" r:id="rId2" location="fishPreservationMethods" xr:uid="{1302D005-C0D4-48F4-9067-8DB21E13C99E}"/>
     <hyperlink ref="M3" r:id="rId3" location="fishPreservationMethods" xr:uid="{EEBE083B-4312-4FA4-A951-C9F9A824B321}"/>
     <hyperlink ref="N3" r:id="rId4" location="fishPreservationMethods" xr:uid="{30064C75-6784-480A-88EC-D543ED3C0DC7}"/>

</xml_diff>